<commit_message>
added SI, EWC, and task incremental code
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DFA52D-1217-194E-A4D7-576F644AF44E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACFFD46-86C7-3D4E-A8A4-7F4041BEDA19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16200" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
+    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -74,43 +74,109 @@
     <t>5-Split MNIST</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>Model</t>
   </si>
   <si>
-    <t>Vanilla BP</t>
-  </si>
-  <si>
-    <t>EIANN w/ BPDale</t>
-  </si>
-  <si>
-    <t>EIANN w/ BTSP</t>
-  </si>
-  <si>
-    <t>EIANN w/ BTSP + ELR</t>
-  </si>
-  <si>
     <t>Expanse</t>
   </si>
   <si>
-    <t>bash optimize_EIANN_frontera_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20240923_nested_optimize_EIANN_2_hidden_CL_mnist_van_bp_relu_SGD_config_G.yaml CL_5split_van_bp</t>
-  </si>
-  <si>
-    <t>bash optimize_EIANN_frontera_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20231129_nested_optimize_EIANN_2_hidden_mnist_CL_bpDale_relu_SGD_config_G.yaml CL_5split_bpDale</t>
-  </si>
-  <si>
-    <t>bash optimize_EIANN_frontera_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20251229_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_config_6L.yaml CL_5split_BTSP</t>
-  </si>
-  <si>
-    <t>EIANN w/ BP_Like</t>
-  </si>
-  <si>
-    <t>bash optimize_EIANN_frontera_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260325_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BP_like_config_5J.yaml CL_5split_BP_Like</t>
-  </si>
-  <si>
-    <t>bash optimize_EIANN_frontera_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260203_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_ELR_config_A.yaml CL_5split_BTSP_ELR</t>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20240923_nested_optimize_EIANN_2_hidden_CL_mnist_van_bp_relu_SGD_config_G.yaml CL_5split_van_bp</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20231129_nested_optimize_EIANN_2_hidden_mnist_CL_bpDale_relu_SGD_config_G.yaml CL_5split_bpDale</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260325_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BP_like_config_5J.yaml CL_5split_BP_Like</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20251229_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_config_6L.yaml CL_5split_BTSP</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260203_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_ELR_config_A.yaml CL_5split_BTSP_ELR</t>
+  </si>
+  <si>
+    <t>COMPLETE</t>
+  </si>
+  <si>
+    <t>Vanilla BP (Task Incremental)</t>
+  </si>
+  <si>
+    <t>Vanilla BP (Class Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale (Class Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BP_Like (Class Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BTSP (Class Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BTSP + ELR (Class Incremental)</t>
+  </si>
+  <si>
+    <t>Vanilla BP + EWC (Class Incremental)</t>
+  </si>
+  <si>
+    <t>Vanilla BP + SI (Class Incremental)</t>
+  </si>
+  <si>
+    <t>Vanilla BP + EWC (Task Incremental)</t>
+  </si>
+  <si>
+    <t>Vanilla BP + SI (Task Incremental)</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_relu_SGD_TI_config_G.yaml CL_5split_van_bp_TI</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260928_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_EWC_relu_SGD_config_A.yaml CL_5split_van_bp_EWC</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260930_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_SI_relu_SGD_config_A.yaml CL_5split_van_bp_SI</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_EWC_relu_SGD_TI_config_A.yaml CL_5split_van_bp_EWC_TI</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_SI_relu_SGD_TI_config_A.yaml CL_5split_van_bp_SI_TI</t>
+  </si>
+  <si>
+    <t>TO DO</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + EWC (Class Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + SI (Class Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + EWC (Task Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + SI (Task Incremental)</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale (Task Incremental)</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260928_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_EWC_config_A.yaml CL_5split_bpDale_EWC</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20260930_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_SI_config_A.yaml CL_5split_bpDale_SI</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_EWC_TI_config_A.yaml CL_5split_bpDale_EWC_TI</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_SI_TI_config_A.yaml CL_5split_bpDale_SI_TI</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_TI_config_G.yaml CL_5split_bpDale_TI</t>
   </si>
 </sst>
 </file>
@@ -490,8 +556,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="208.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -515,10 +581,10 @@
         <v>7</v>
       </c>
       <c r="G1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H1" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="I1" t="s">
         <v>3</v>
@@ -532,7 +598,7 @@
         <v>46282</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -544,10 +610,13 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
         <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -558,7 +627,7 @@
         <v>46282</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -570,10 +639,13 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
         <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -584,7 +656,7 @@
         <v>46282</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -596,10 +668,13 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -610,7 +685,7 @@
         <v>46282</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
         <v>6</v>
@@ -622,10 +697,13 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
+        <v>18</v>
       </c>
       <c r="I5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -636,22 +714,315 @@
         <v>46282</v>
       </c>
       <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" t="s">
-        <v>23</v>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" t="s">
+        <v>19</v>
+      </c>
+      <c r="H9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" t="s">
+        <v>35</v>
+      </c>
+      <c r="I10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" t="s">
+        <v>39</v>
+      </c>
+      <c r="H16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="5:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
added TI learning for EI networks
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACFFD46-86C7-3D4E-A8A4-7F4041BEDA19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35AAE247-545C-A246-ACFE-2383EF485AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261001_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_TI_config_G.yaml CL_5split_bpDale_TI</t>
+  </si>
+  <si>
+    <t>RUNNING</t>
   </si>
 </sst>
 </file>
@@ -758,7 +761,7 @@
         <v>25</v>
       </c>
       <c r="H7" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="I7" t="s">
         <v>31</v>
@@ -787,7 +790,7 @@
         <v>26</v>
       </c>
       <c r="H8" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="I8" t="s">
         <v>32</v>
@@ -816,7 +819,7 @@
         <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="I9" t="s">
         <v>30</v>
@@ -845,7 +848,7 @@
         <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="I10" t="s">
         <v>33</v>
@@ -874,7 +877,7 @@
         <v>28</v>
       </c>
       <c r="H11" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="I11" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
added btsp_bp learning rules
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA519A0-0619-284C-A3BF-CDBCC1C6C49E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162B911D-AA9F-F042-9801-9274BAB3211A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="-18900" windowWidth="28800" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="63">
   <si>
     <t>Date</t>
   </si>
@@ -195,6 +195,39 @@
   </si>
   <si>
     <t>nested.analyze of all completed CI Runs</t>
+  </si>
+  <si>
+    <t>STOPPED</t>
+  </si>
+  <si>
+    <t>Inefficient memory  allocation</t>
+  </si>
+  <si>
+    <t>ENDED</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + SI (Class Incremental) Hot Start</t>
+  </si>
+  <si>
+    <t>EIANN w/DTP + SI (Class Incremental) Hot Start</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist_hot_start.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20260930_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_SI_config_A.yaml CL_5split_bpDale_SI /expanse/lustre/scratch/rpemmaraju/temp_project/data/EIANN/20261005_105117_nested_optimization_history_PopulationAnnealing_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_SI_A_124562835820294074569634942619043933184.hdf5</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist_hot_start.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261002_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_DTP_SI_config_5J.yaml CL_5split_DTP_SI  /expanse/lustre/scratch/rpemmaraju/temp_project/data/EIANN/20261005_105054_nested_optimization_history_PopulationAnnealing_EIANN_2_hidden_CL_mnist_5_tasks_DTP_SI_5J_106496651045923541041349860333180857984.hdf5</t>
+  </si>
+  <si>
+    <t>OOM</t>
+  </si>
+  <si>
+    <t>OOM -&gt; adding more memory for HS</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + EWC (Class Incremental) Hot Start</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist_hot_start.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20260928_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_EWC_config_A.yaml CL_5split_bpDale_EWC /expanse/lustre/scratch/rpemmaraju/temp_project/data/EIANN/20261006_090235_nested_optimization_history_PopulationAnnealing_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_EWC_A_117784733731023246787354137130969510408.hdf5</t>
   </si>
 </sst>
 </file>
@@ -567,13 +600,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BA0BB30-FCFB-F74F-BDE2-526FA9424698}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="208.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -954,7 +987,7 @@
         <v>36</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J13" t="s">
         <v>38</v>
@@ -983,7 +1016,7 @@
         <v>39</v>
       </c>
       <c r="H14" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J14" t="s">
         <v>40</v>
@@ -1041,7 +1074,7 @@
         <v>43</v>
       </c>
       <c r="H16" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="I16" t="s">
         <v>49</v>
@@ -1105,10 +1138,7 @@
         <v>35</v>
       </c>
       <c r="H18" t="s">
-        <v>45</v>
-      </c>
-      <c r="I18" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="J18" t="s">
         <v>37</v>
@@ -1119,7 +1149,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="1">
-        <v>46295</v>
+        <v>46302</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -1137,11 +1167,261 @@
         <v>51</v>
       </c>
       <c r="H19" t="s">
-        <v>45</v>
+        <v>52</v>
+      </c>
+      <c r="I19" t="s">
+        <v>53</v>
       </c>
       <c r="J19" t="s">
         <v>50</v>
       </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46302</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" t="s">
+        <v>18</v>
+      </c>
+      <c r="J20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46303</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" t="s">
+        <v>55</v>
+      </c>
+      <c r="H21" t="s">
+        <v>46</v>
+      </c>
+      <c r="I21" t="s">
+        <v>59</v>
+      </c>
+      <c r="J21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46303</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" t="s">
+        <v>56</v>
+      </c>
+      <c r="H22" t="s">
+        <v>46</v>
+      </c>
+      <c r="I22" t="s">
+        <v>59</v>
+      </c>
+      <c r="J22" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46304</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" t="s">
+        <v>46</v>
+      </c>
+      <c r="I23" t="s">
+        <v>60</v>
+      </c>
+      <c r="J23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="1">
+        <v>46304</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" t="s">
+        <v>56</v>
+      </c>
+      <c r="H24" t="s">
+        <v>46</v>
+      </c>
+      <c r="I24" t="s">
+        <v>59</v>
+      </c>
+      <c r="J24" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46304</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" t="s">
+        <v>55</v>
+      </c>
+      <c r="H25" t="s">
+        <v>18</v>
+      </c>
+      <c r="J25" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46304</v>
+      </c>
+      <c r="C26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" t="s">
+        <v>56</v>
+      </c>
+      <c r="H26" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46305</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" t="s">
+        <v>61</v>
+      </c>
+      <c r="H27" t="s">
+        <v>45</v>
+      </c>
+      <c r="J27" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B28" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added BTSP + SI
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162B911D-AA9F-F042-9801-9274BAB3211A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5894B9EA-4698-034C-A2E4-C821487B7656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="-18900" windowWidth="28800" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="67">
   <si>
     <t>Date</t>
   </si>
@@ -228,6 +228,18 @@
   </si>
   <si>
     <t>bash optimize_EIANN_expanse_cpu_mnist_hot_start.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20260928_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_EWC_config_A.yaml CL_5split_bpDale_EWC /expanse/lustre/scratch/rpemmaraju/temp_project/data/EIANN/20261006_090235_nested_optimization_history_PopulationAnnealing_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_EWC_A_117784733731023246787354137130969510408.hdf5</t>
+  </si>
+  <si>
+    <t>EIANN w/ BTSP_BP</t>
+  </si>
+  <si>
+    <t>EIANN w/ BTSP_BP + ELR</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261012_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_BP_config_A.yaml CL_5split_BTSP_BP</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/20261012_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_ELR_BP_config_A.yaml CL_5split_BTSP_ELR_BP</t>
   </si>
 </sst>
 </file>
@@ -600,7 +612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BA0BB30-FCFB-F74F-BDE2-526FA9424698}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
@@ -1414,14 +1426,69 @@
         <v>61</v>
       </c>
       <c r="H27" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="J27" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B28" s="1"/>
+      <c r="A28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" s="1">
+        <v>46307</v>
+      </c>
+      <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>6</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H28" t="s">
+        <v>45</v>
+      </c>
+      <c r="J28" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="1">
+        <v>46307</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" t="s">
+        <v>64</v>
+      </c>
+      <c r="H29" t="s">
+        <v>45</v>
+      </c>
+      <c r="J29" t="s">
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
increased nodes for job
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239904C7-7005-D84D-84EE-6C56ED31DD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC6ACCD-579F-ED40-B51D-0BC80B5079ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="-18900" windowWidth="28800" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261014_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_SI_ELR_config_A.yaml CL_5split_bpDale_SI_ELR</t>
+  </si>
+  <si>
+    <t>Vanilla BP + SI Hypergradient (Class Incremental)</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261014_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_SI_HD_relu_SGD_config_A.yaml CL_5split_bpDale_SI_HG</t>
   </si>
 </sst>
 </file>
@@ -630,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BA0BB30-FCFB-F74F-BDE2-526FA9424698}">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
@@ -1601,6 +1607,102 @@
         <v>72</v>
       </c>
     </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" t="s">
+        <v>6</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" t="s">
+        <v>69</v>
+      </c>
+      <c r="H33" t="s">
+        <v>46</v>
+      </c>
+      <c r="I33" t="s">
+        <v>59</v>
+      </c>
+      <c r="J33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B34" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C34" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" t="s">
+        <v>71</v>
+      </c>
+      <c r="H34" t="s">
+        <v>46</v>
+      </c>
+      <c r="I34" t="s">
+        <v>59</v>
+      </c>
+      <c r="J34" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B35" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C35" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" t="s">
+        <v>6</v>
+      </c>
+      <c r="E35" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35" t="s">
+        <v>73</v>
+      </c>
+      <c r="H35" t="s">
+        <v>46</v>
+      </c>
+      <c r="I35" t="s">
+        <v>59</v>
+      </c>
+      <c r="J35" t="s">
+        <v>74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
addressed memory issue in batch scripts
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC6ACCD-579F-ED40-B51D-0BC80B5079ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7017144-F90D-184B-8892-01699267C8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-18900" windowWidth="28800" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
+    <workbookView xWindow="0" yWindow="1140" windowWidth="28800" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="81">
   <si>
     <t>Date</t>
   </si>
@@ -264,6 +264,24 @@
   </si>
   <si>
     <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261014_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_SI_HD_relu_SGD_config_A.yaml CL_5split_bpDale_SI_HG</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist_hot_start.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261013_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_SI_config_6L.yaml CL_5split_BTSP_SI /expanse/lustre/scratch/rpemmaraju/temp_project/data/EIANN/20261013_120509_nested_optimization_history_PopulationAnnealing_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_SI_6L_3696222178511307923271926805588798446.hdf5</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist_hot_start.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261012_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_ELR_BP_config_A.yaml CL_5split_BTSP_ELR_BP /expanse/lustre/scratch/rpemmaraju/temp_project/data/EIANN/20261013_105259_nested_optimization_history_PopulationAnnealing_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_ELR_BP_A_316274938518758798260530043048878580016.hdf5</t>
+  </si>
+  <si>
+    <t>OOM -&gt; adding more train memory</t>
+  </si>
+  <si>
+    <t>EIANN w/ BTSP_BP + ELR (Class Incremental) Hot Start</t>
+  </si>
+  <si>
+    <t>EIANN w/ BTSP + SI (Class Incremental) Hot Start</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261014_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_SI_HD_relu_SGD_config_A.yaml CL_5split_van_bp_SI_HG</t>
   </si>
 </sst>
 </file>
@@ -636,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BA0BB30-FCFB-F74F-BDE2-526FA9424698}">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
@@ -1479,7 +1497,7 @@
         <v>66</v>
       </c>
       <c r="H28" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="J28" t="s">
         <v>64</v>
@@ -1508,7 +1526,7 @@
         <v>67</v>
       </c>
       <c r="H29" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J29" t="s">
         <v>63</v>
@@ -1537,7 +1555,7 @@
         <v>65</v>
       </c>
       <c r="H30" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J30" t="s">
         <v>68</v>
@@ -1697,10 +1715,184 @@
         <v>46</v>
       </c>
       <c r="I35" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="J35" t="s">
         <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>5</v>
+      </c>
+      <c r="B36" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>6</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H36" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>6</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37" t="s">
+        <v>78</v>
+      </c>
+      <c r="H37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J37" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>5</v>
+      </c>
+      <c r="B38" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>6</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" t="s">
+        <v>69</v>
+      </c>
+      <c r="H38" t="s">
+        <v>45</v>
+      </c>
+      <c r="J38" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>5</v>
+      </c>
+      <c r="B39" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>6</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>10</v>
+      </c>
+      <c r="G39" t="s">
+        <v>71</v>
+      </c>
+      <c r="H39" t="s">
+        <v>45</v>
+      </c>
+      <c r="J39" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>5</v>
+      </c>
+      <c r="B40" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>6</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" t="s">
+        <v>73</v>
+      </c>
+      <c r="H40" t="s">
+        <v>46</v>
+      </c>
+      <c r="I40" t="s">
+        <v>59</v>
+      </c>
+      <c r="J40" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>6</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" t="s">
+        <v>73</v>
+      </c>
+      <c r="J41" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made validation batched and added BTSP_SI_HD
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/runs.xlsx
+++ b/runs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rahul/Documents/Milstein_lab/EIANN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3774DA6F-1BF9-1D4A-965F-8FF2CE02FF31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20729CC5-5384-C549-A15C-DD134FAF21D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="-18900" windowWidth="28800" windowHeight="16180" xr2:uid="{A618CDC5-8790-0244-82CF-43BDF0E1892F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="89">
   <si>
     <t>Date</t>
   </si>
@@ -290,6 +290,9 @@
     <t>Vanilla BP + SI Hypergradient_v1 (Class Incremental)</t>
   </si>
   <si>
+    <t>RUNNING</t>
+  </si>
+  <si>
     <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261021_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_van_bp_SI_HD_v1_relu_SGD_config_A.yaml CL_5split_van_bp_SI_HG_v1</t>
   </si>
   <si>
@@ -297,6 +300,12 @@
   </si>
   <si>
     <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261021_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_BTSP_SI_layer_lambda_config_6L.yaml CL_5split_BTSP_SI</t>
+  </si>
+  <si>
+    <t>EIANN w/ BPDale + SI Hypergradient_v1 (Class Incremental)</t>
+  </si>
+  <si>
+    <t>bash optimize_EIANN_expanse_cpu_mnist.sh /expanse/lustre/projects/sua199/rpemmaraju/EIANN/EIANN/optimize/optimize_config/mnist_CL/5_tasks/20261021_nested_optimize_EIANN_2_hidden_CL_mnist_5_tasks_bpDale_relu_SGD_SI_HD_v1_config_A.yaml CL_5split_bpDale_SI_HG_v1</t>
   </si>
 </sst>
 </file>
@@ -669,12 +678,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BA0BB30-FCFB-F74F-BDE2-526FA9424698}">
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="50.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="208.5" bestFit="1" customWidth="1"/>
   </cols>
@@ -1935,8 +1944,11 @@
       <c r="G42" t="s">
         <v>82</v>
       </c>
+      <c r="H42" t="s">
+        <v>18</v>
+      </c>
       <c r="J42" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
@@ -1961,11 +1973,43 @@
       <c r="G43" t="s">
         <v>64</v>
       </c>
+      <c r="H43" t="s">
+        <v>18</v>
+      </c>
       <c r="I43" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J43" t="s">
-        <v>85</v>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>5</v>
+      </c>
+      <c r="B44" s="1">
+        <v>46310</v>
+      </c>
+      <c r="C44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D44" t="s">
+        <v>6</v>
+      </c>
+      <c r="E44" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" t="s">
+        <v>10</v>
+      </c>
+      <c r="G44" t="s">
+        <v>87</v>
+      </c>
+      <c r="H44" t="s">
+        <v>83</v>
+      </c>
+      <c r="J44" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>